<commit_message>
feat: Implement semester promotion for class students
- Added functionality to promote all students in a class to the next semester for teachers and admins.
- Created a new API endpoint to handle semester promotion requests.
- Updated the class and user models to reflect the changes in semester.
- Enhanced the ManageUsers component to filter users by semester.
- Updated tests to cover the new promotion feature and ensure proper access control.
- Refactored console logs to use a consistent logging format across the application.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/bulk-student-import-sample.xlsx
+++ b/frontend/public/templates/bulk-student-import-sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University files\Programming\MERN Projects\AttendX\AttendX\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573BA157-C4A4-4466-A174-D7AE59C02760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E71F6C-6818-458E-9662-026CD7B8CD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>name</t>
   </si>
@@ -76,9 +76,6 @@
     <t>EEE-2403</t>
   </si>
   <si>
-    <t>EEE</t>
-  </si>
-  <si>
     <t>2022-2026</t>
   </si>
   <si>
@@ -98,36 +95,6 @@
   </si>
   <si>
     <t>CS</t>
-  </si>
-  <si>
-    <t>BBA</t>
-  </si>
-  <si>
-    <t>BCA</t>
-  </si>
-  <si>
-    <t>ECE</t>
-  </si>
-  <si>
-    <t>ME</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>MBA</t>
-  </si>
-  <si>
-    <t>MCA</t>
-  </si>
-  <si>
-    <t>Biotechnology</t>
-  </si>
-  <si>
-    <t>Commerce</t>
-  </si>
-  <si>
-    <t>Economics</t>
   </si>
   <si>
     <t>Password123</t>
@@ -519,8 +486,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.796875" customWidth="1"/>
     <col min="2" max="2" width="30.796875" customWidth="1"/>
@@ -533,7 +500,7 @@
     <col min="9" max="9" width="10.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -562,15 +529,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -582,7 +549,7 @@
         <v>5</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
         <v>12</v>
@@ -591,15 +558,15 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
@@ -611,7 +578,7 @@
         <v>5</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H3" t="s">
         <v>12</v>
@@ -620,15 +587,15 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>17</v>
@@ -640,71 +607,48 @@
         <v>4</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I4">
         <v>2024</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G5" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G6" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G8" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G9" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G10" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G11" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G12" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G13" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G14" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="G15" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G15" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>